<commit_message>
Nap anh minh chung that (76 anh, 17 su kien), carousel logo header, tai lieu du an
Nen anh HEIC/JPG goc (toi 18MB/anh) qua Pillow+pillow-heif xuong duoi 1MB,
ghep vao content/events/*.json theo ghi chu trong mau-nhap-hoat-dong.xlsx.
Them carousel truot ngang o vi tri logo dau trang (huy hieu + 15 anh
Banner, 2 giay/anh, lap vo han). Cap nhat PROJECT.md, tao VIDEO-PRODUCTION.md
tach rieng trang thai video du thi - tu phien nay cap nhat docs/ ngay sau
moi nhiem vu.
</commit_message>
<xml_diff>
--- a/uploads/mau-nhap-hoat-dong.xlsx
+++ b/uploads/mau-nhap-hoat-dong.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{717425BC-9FC3-4944-A341-99C08D32AEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66085B92-BC87-4F9F-A5F9-DABB98EE2CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nhap hoat dong" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="119">
   <si>
     <t>STT</t>
   </si>
@@ -207,6 +207,177 @@
   </si>
   <si>
     <t>Tuyên truyền, phổ biến, giáo dục pháp luật, hướng dẫn sử dụng Internet và mạng xã hội an toàn, hiệu quả, đúng pháp luật cho học sinh trường THPT Nguyễn Thị Minh Khai, Quận Bắc Từ Liêm, TP Hà Nội</t>
+  </si>
+  <si>
+    <t>Trường Liên cấp THCS, Tiểu học tư thục Ngôi Sao Hà Nội</t>
+  </si>
+  <si>
+    <t>Các kiến thức, kỹ năm về phòng, chống lừa đảo, "bắt cóc online", xâm hại tình dục và phòng, chống các hành vi vi phạm pháp luật khác trên không gian mạng</t>
+  </si>
+  <si>
+    <t>Trường THCS Phan Chu Trinh, phường Giảng Võ, TP Hà Nội</t>
+  </si>
+  <si>
+    <t>Các kiến thức, kỹ năm về an ninh, an toàn trên không gian mạng, sử dụng Internet an toàn, phòng tránh bắt cóc trực tuyến, phòng tránh lửa đảo trên không gian mạng</t>
+  </si>
+  <si>
+    <t>Trường THCS và THPT Marie Curie</t>
+  </si>
+  <si>
+    <t>Các kiến thức, kỹ năm bảo đảm an ninh, an toàn khi sử dụng mạng Internet, mạng xã hội, các kiến thức phòng, chống lừa đảo, "bắt cóc online", xâm hại tình dục và phòng, chống các hành vi vi phạm pháp luật khác trên không gian mạng</t>
+  </si>
+  <si>
+    <t>An ninh, an toàn trên không gian mạng cho học sinh nhà trường</t>
+  </si>
+  <si>
+    <t>Trường THCS và THPT Marie Curie Long Biên</t>
+  </si>
+  <si>
+    <t>Kỹ năng đảm bảo an ninh, an toàn trên không gian mạng</t>
+  </si>
+  <si>
+    <t>Trường THCS Giảng Võ, phường Giảng Võ, TP Hà Nội</t>
+  </si>
+  <si>
+    <t>Các kiến thức, kỹ năng về an ninh, an toàn trên không gian mạng, sử dụng internet an toàn, phòng tránh bắt cóc trực tuyến, phòng tránh lừa đảo trên không gian mạng cho học sinh</t>
+  </si>
+  <si>
+    <t>Trường THCS Nguyễn Trãi, phường Giảng Võ, TP Hà Nội</t>
+  </si>
+  <si>
+    <t>Chuyên đề pháp luật vè an ninh mạng, sử dụng Internet an toàn cho học sinh của nhà trường</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trường Tiểu học Đoàn Thị Điểm </t>
+  </si>
+  <si>
+    <t>Các kiến thức, kỹ năng cần thiết để tự bảo vệ bản thân khi tham gia môi trường mạng (nhận biết thông tin xấu độc, bảo mật tài khoản, phòng tránh lừa đảo trực tuyến, phòng tránh nguy cơ bị bắt cóc, xâm hại, sử dụng dịch vụ xe công nghệ an toàn,…)</t>
+  </si>
+  <si>
+    <t>Trường Tiểu học Đoàn Thị Điểm (Symphony) - Hà Nội</t>
+  </si>
+  <si>
+    <t>Em an toàn mọi lúc, mọi nơi</t>
+  </si>
+  <si>
+    <t>Trường Phổ thông Dân tộc bán trú Tiểu học Vừ A Dính, thôn Có Thái, xã Nậm Có, tỉnh Lào Cai</t>
+  </si>
+  <si>
+    <t>An toàn thông tin - Kỹ năng cần thiết cho học sinh tiểu học</t>
+  </si>
+  <si>
+    <t>Uỷ ban Mặt trận Tổ quốc Việt Nam phường Xuân Đỉnh, TP Hà Nội</t>
+  </si>
+  <si>
+    <t>Tuyên truyền pháp luật về an ninh mạng; phổ biến, hướng dẫn sử dụng Internet, mạng xã hội an toàn, văn minh, đúng pháp luật và cách bảo mật thông tin các nhân trên Internet</t>
+  </si>
+  <si>
+    <t>Trường Tiểu học Trung Tự, phường Kim Liên, TP Hà Nội</t>
+  </si>
+  <si>
+    <t>Em an toàn trên môi trường mạng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://hvcsnd.edu.vn/tuyen-truyen-trang-bi-ky-nang-su-dung-mang-xa-hoi-an-toan-cho-hoc-sinh-truong-thcs-xuan-truong-nam-dinh-12636 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://hvcsnd.edu.vn/tuyen-truyen-huong-dan-su-dung-internet-va-giao-tiep-ung-xu-tren-khong-gian-mang-11869 </t>
+  </si>
+  <si>
+    <t>https://hvcsnd.edu.vn/khoa-toan-tin-hoc-va-ung-dung-khcn-trong-pctp-tuyen-truyen-pho-bien-giao-duc-phap-luat-cho-hoc-sinh-tai-ha-noi-11252</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://hvcsnd.edu.vn/khoa-toan-tin-hoc-va-ung-dung-khcn-trong-pctp-tuyen-truyen-pho-bien-giao-duc-phap-luat-cho-hoc-sinh-tai-ha-noi-11252 </t>
+  </si>
+  <si>
+    <t>Trường THCS Phúc Diễn</t>
+  </si>
+  <si>
+    <t>Thiện nguyện</t>
+  </si>
+  <si>
+    <t>Tuyên truyền sử dụng mạng xã hội an toàn, có hiệu quả vì một môi trường mạng xã hội bình yên</t>
+  </si>
+  <si>
+    <t>15,16/11/2024</t>
+  </si>
+  <si>
+    <t>2 điểm trường Pa Cốp và Gốc Đa của trường Tiểu học Vân Hồ, xã Vân Hồ, huyện Vân Hồ, tỉnh Sơn La</t>
+  </si>
+  <si>
+    <t>Trường Tiểu học và THCS Vần Dính, xã Thượng Thôn, huyện Quảng Hà, tỉnh Cao Bằng</t>
+  </si>
+  <si>
+    <t>02,03/02/2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ngoisaohanoi.edu.vn/ngoi-sao-ha-noi-chu-dong-trang-bi-la-chan-an-toan-cho-hansers-khoi-trung-hoc-co-so/ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://c2giangvo2.giangvo.edu.vn/chi-tiet/truong-thcs-giang-vo-2-to-chuc-tuyen-truyen-an-toa-pmtd22sw25208 </t>
+  </si>
+  <si>
+    <t>An toàn, an ninh mạng</t>
+  </si>
+  <si>
+    <t>Trường THCS Giảng Võ 2, TP Hà Nội</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://hvcsnd.edu.vn/hanh-trinh-se-chia-yeu-thuong-tai-truong-pho-thong-dan-toc-ban-tru-tieu-hoc-vu-a-dinh-xa-nam-co-tinh-lao-cai-13680 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://hn-ams.edu.vn/en/node/39102 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://hvcsnd.edu.vn/tuyen-truyen-pho-bien-giao-duc-phap-luat-huong-dan-su-dung-internet-va-mang-xa-hoi-an-toan-hieu-qua-11155 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://anninhthudo.vn/tuyen-truyen-su-dung-internet-mang-xa-hoi-an-toan-cho-hoc-sinh-post627307.antd </t>
+  </si>
+  <si>
+    <t>Có 3 ảnh ở C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Vần dính</t>
+  </si>
+  <si>
+    <t>Có 2 ảnh ở C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Pacop</t>
+  </si>
+  <si>
+    <t>Có 3 ảnh ở C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Vừ a dính</t>
+  </si>
+  <si>
+    <t>Có 11 ảnh ở thư mục C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Nguyễn Thị Minh Khai</t>
+  </si>
+  <si>
+    <t>Có 6 ảnh ở thư mục C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Hà Nội Arm</t>
+  </si>
+  <si>
+    <t>Có 6 ảnh ở C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Cầu giấy 2</t>
+  </si>
+  <si>
+    <t>Có 2 ảnh ở C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Thượng cát</t>
+  </si>
+  <si>
+    <t>Có 6 ảnh ở thư mục C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Cầu giấy</t>
+  </si>
+  <si>
+    <t>Có 4 ảnh ở C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Xuân Đỉnh</t>
+  </si>
+  <si>
+    <t>Có 4 ảnh ở C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Ngôi sao Hà Nội</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/share/p/1SE5BUFGcc/</t>
+  </si>
+  <si>
+    <t>Có 10 ảnh ở C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Marie Curie</t>
+  </si>
+  <si>
+    <t>Có 8 ảnh ở C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Đoàn Thị Điểm</t>
+  </si>
+  <si>
+    <t>https://hvcsnd.edu.vn/hoc-vien-csnd-phoi-hop-truong-thcs-tran-duy-hung-to-chuc-chuong-trinh-em-an-toan-tren-moi-truong-mang-13270</t>
+  </si>
+  <si>
+    <t>Có 3 ảnh ở C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\Mai Dịch</t>
   </si>
 </sst>
 </file>
@@ -308,7 +479,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -370,25 +541,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -434,17 +592,20 @@
     <xf numFmtId="14" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -750,7 +911,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" style="6" customWidth="1"/>
@@ -758,7 +919,7 @@
     <col min="3" max="3" width="18" style="6" customWidth="1"/>
     <col min="4" max="4" width="27.77734375" style="6" customWidth="1"/>
     <col min="5" max="5" width="16" style="6" customWidth="1"/>
-    <col min="6" max="6" width="34.44140625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="52" style="6" customWidth="1"/>
     <col min="7" max="7" width="46" style="6" customWidth="1"/>
     <col min="8" max="10" width="30" style="6" customWidth="1"/>
     <col min="11" max="16384" width="8.77734375" style="6"/>
@@ -826,242 +987,294 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="43.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="82.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
         <v>1</v>
       </c>
-      <c r="B3" s="9"/>
+      <c r="B3" s="9" t="s">
+        <v>90</v>
+      </c>
       <c r="C3" s="9" t="s">
         <v>32</v>
       </c>
       <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
+      <c r="E3" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>94</v>
+      </c>
       <c r="G3" s="9"/>
       <c r="H3" s="10" t="s">
         <v>29</v>
       </c>
       <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-    </row>
-    <row r="4" spans="1:10" ht="43.95" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J3" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="76.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8">
         <v>2</v>
       </c>
-      <c r="B4" s="9"/>
+      <c r="B4" s="9" t="s">
+        <v>90</v>
+      </c>
       <c r="C4" s="9" t="s">
         <v>32</v>
       </c>
       <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
+      <c r="E4" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>93</v>
+      </c>
       <c r="G4" s="9"/>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="22" t="s">
         <v>30</v>
       </c>
       <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-    </row>
-    <row r="5" spans="1:10" ht="43.95" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J4" s="9" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="102" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="8">
         <v>3</v>
       </c>
-      <c r="B5" s="9"/>
+      <c r="B5" s="9" t="s">
+        <v>90</v>
+      </c>
       <c r="C5" s="9" t="s">
         <v>32</v>
       </c>
       <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
+      <c r="E5" s="12">
+        <v>46017</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>79</v>
+      </c>
       <c r="G5" s="9"/>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="22" t="s">
         <v>31</v>
       </c>
       <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-    </row>
-    <row r="6" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J5" s="9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="99" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9" t="s">
-        <v>60</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="9"/>
       <c r="E6" s="12">
-        <v>44788</v>
+        <v>44285</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
+      <c r="H6" s="22" t="s">
+        <v>29</v>
+      </c>
       <c r="I6" s="9"/>
       <c r="J6" s="9"/>
     </row>
     <row r="7" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="E7" s="16">
-        <v>44839</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>51</v>
+      <c r="D7" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" s="12">
+        <v>44788</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>59</v>
       </c>
       <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
+      <c r="H7" s="20" t="s">
+        <v>102</v>
+      </c>
       <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
+      <c r="J7" s="9" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="8" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E8" s="19">
-        <v>44841</v>
-      </c>
-      <c r="F8" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" s="14"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
+      <c r="C8" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="16">
+        <v>44839</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="9"/>
+      <c r="H8" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="I8" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="9" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="17">
+        <v>44841</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" s="14"/>
+      <c r="H9" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="8">
+        <v>8</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C9" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="C10" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E10" s="17">
         <v>44875</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="F10" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="G9" s="14"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-    </row>
-    <row r="10" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="8"/>
-      <c r="B10" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E10" s="19">
-        <v>44881</v>
-      </c>
-      <c r="F10" s="20" t="s">
-        <v>56</v>
-      </c>
       <c r="G10" s="14"/>
-      <c r="H10" s="11"/>
+      <c r="H10" s="21" t="s">
+        <v>88</v>
+      </c>
       <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
+      <c r="J10" s="9" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="11" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" s="19">
-        <v>45167</v>
-      </c>
-      <c r="F11" s="20" t="s">
-        <v>34</v>
+        <v>57</v>
+      </c>
+      <c r="E11" s="17">
+        <v>44881</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>56</v>
       </c>
       <c r="G11" s="14"/>
-      <c r="H11" s="9"/>
+      <c r="H11" s="11"/>
       <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
+      <c r="J11" s="9" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="12" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="8">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="19">
-        <v>45189</v>
-      </c>
-      <c r="F12" s="20" t="s">
-        <v>46</v>
+        <v>33</v>
+      </c>
+      <c r="E12" s="17">
+        <v>45167</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>34</v>
       </c>
       <c r="G12" s="14"/>
-      <c r="H12" s="9"/>
+      <c r="H12" s="20" t="s">
+        <v>86</v>
+      </c>
       <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
+      <c r="J12" s="9" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="13" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="8">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="21">
-        <v>45208</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>37</v>
+        <v>47</v>
+      </c>
+      <c r="E13" s="17">
+        <v>45189</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>46</v>
       </c>
       <c r="G13" s="14"/>
       <c r="H13" s="9"/>
@@ -1070,159 +1283,249 @@
     </row>
     <row r="14" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="8">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C14" s="13" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="E14" s="21">
-        <v>45432</v>
+        <v>36</v>
+      </c>
+      <c r="E14" s="19">
+        <v>45208</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G14" s="14"/>
-      <c r="H14" s="9"/>
+      <c r="H14" s="9" t="s">
+        <v>117</v>
+      </c>
       <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
+      <c r="J14" s="9" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="15" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="8">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E15" s="21">
-        <v>45597</v>
+        <v>38</v>
+      </c>
+      <c r="E15" s="19">
+        <v>45432</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G15" s="14"/>
-      <c r="H15" s="9"/>
+      <c r="H15" s="9" t="s">
+        <v>117</v>
+      </c>
       <c r="I15" s="9"/>
       <c r="J15" s="9"/>
     </row>
     <row r="16" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="8">
-        <v>12</v>
-      </c>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
+        <v>14</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="19">
+        <v>45597</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" s="14"/>
+      <c r="H16" s="20" t="s">
+        <v>85</v>
+      </c>
       <c r="I16" s="9"/>
       <c r="J16" s="9"/>
     </row>
-    <row r="17" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" ht="52.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="8">
-        <v>9</v>
-      </c>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
+        <v>15</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
+      <c r="E17" s="12">
+        <v>45940</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>62</v>
+      </c>
       <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
+      <c r="H17" s="20" t="s">
+        <v>96</v>
+      </c>
       <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-    </row>
-    <row r="18" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J17" s="9" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="55.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="8">
-        <v>10</v>
-      </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
+        <v>16</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
+      <c r="E18" s="12">
+        <v>45946</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>64</v>
+      </c>
       <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
+      <c r="H18" s="20" t="s">
+        <v>103</v>
+      </c>
       <c r="I18" s="9"/>
       <c r="J18" s="9"/>
     </row>
     <row r="19" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="8">
-        <v>11</v>
-      </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
+        <v>17</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
+      <c r="E19" s="12">
+        <v>45955</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>66</v>
+      </c>
       <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
+      <c r="H19" s="20" t="s">
+        <v>114</v>
+      </c>
       <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
+      <c r="J19" s="9" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="20" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="8">
-        <v>12</v>
-      </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
+        <v>18</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
+      <c r="E20" s="12">
+        <v>45965</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>66</v>
+      </c>
       <c r="G20" s="9"/>
       <c r="H20" s="9"/>
       <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
+      <c r="J20" s="9" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="21" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="8">
-        <v>13</v>
-      </c>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
+        <v>19</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
+      <c r="E21" s="12">
+        <v>45966</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>66</v>
+      </c>
       <c r="G21" s="9"/>
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
+      <c r="J21" s="9" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="22" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="8">
-        <v>14</v>
-      </c>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
+        <v>20</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
+      <c r="E22" s="12">
+        <v>46017</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>69</v>
+      </c>
       <c r="G22" s="9"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
+      <c r="J22" s="9" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="23" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="8">
-        <v>15</v>
-      </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
+        <v>21</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
+      <c r="E23" s="12">
+        <v>45957</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>71</v>
+      </c>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
@@ -1230,13 +1533,21 @@
     </row>
     <row r="24" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="8">
-        <v>16</v>
-      </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
+        <v>22</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
+      <c r="E24" s="12">
+        <v>45968</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>73</v>
+      </c>
       <c r="G24" s="9"/>
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
@@ -1244,13 +1555,21 @@
     </row>
     <row r="25" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="8">
-        <v>17</v>
-      </c>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
+        <v>23</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
+      <c r="E25" s="12">
+        <v>45968</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>83</v>
+      </c>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
@@ -1258,77 +1577,125 @@
     </row>
     <row r="26" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="8">
-        <v>18</v>
-      </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
+        <v>24</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
+      <c r="E26" s="12">
+        <v>45978</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>75</v>
+      </c>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
+      <c r="J26" s="9" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="27" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="8">
-        <v>19</v>
-      </c>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
+        <v>25</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
+      <c r="E27" s="12">
+        <v>45985</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>77</v>
+      </c>
       <c r="G27" s="9"/>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-    </row>
-    <row r="28" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J27" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="73.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="8">
-        <v>20</v>
-      </c>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
+        <v>26</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
+      <c r="E28" s="12">
+        <v>46017</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>79</v>
+      </c>
       <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
+      <c r="H28" s="21" t="s">
+        <v>100</v>
+      </c>
       <c r="I28" s="9"/>
       <c r="J28" s="9"/>
     </row>
     <row r="29" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8">
-        <v>21</v>
-      </c>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9"/>
+        <v>27</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
+      <c r="E29" s="12">
+        <v>46038</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>81</v>
+      </c>
       <c r="G29" s="9"/>
       <c r="H29" s="9"/>
       <c r="I29" s="9"/>
       <c r="J29" s="9"/>
     </row>
-    <row r="30" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" ht="46.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="8">
-        <v>22</v>
-      </c>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
+        <v>28</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
+      <c r="E30" s="12">
+        <v>46112</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>99</v>
+      </c>
       <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
+      <c r="H30" s="20" t="s">
+        <v>97</v>
+      </c>
       <c r="I30" s="9"/>
       <c r="J30" s="9"/>
     </row>
     <row r="31" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="8">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
@@ -1342,7 +1709,7 @@
     </row>
     <row r="32" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="8">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -1354,93 +1721,9 @@
       <c r="I32" s="9"/>
       <c r="J32" s="9"/>
     </row>
-    <row r="33" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="8">
-        <v>25</v>
-      </c>
-      <c r="B33" s="9"/>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-      <c r="G33" s="9"/>
-      <c r="H33" s="9"/>
-      <c r="I33" s="9"/>
-      <c r="J33" s="9"/>
-    </row>
-    <row r="34" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="8">
-        <v>26</v>
-      </c>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
-      <c r="I34" s="9"/>
-      <c r="J34" s="9"/>
-    </row>
-    <row r="35" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="8">
-        <v>27</v>
-      </c>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="9"/>
-    </row>
-    <row r="36" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="8">
-        <v>28</v>
-      </c>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="9"/>
-      <c r="J36" s="9"/>
-    </row>
-    <row r="37" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="8">
-        <v>29</v>
-      </c>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
-      <c r="H37" s="9"/>
-      <c r="I37" s="9"/>
-      <c r="J37" s="9"/>
-    </row>
-    <row r="38" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="8">
-        <v>30</v>
-      </c>
-      <c r="B38" s="9"/>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="9"/>
-      <c r="I38" s="9"/>
-      <c r="J38" s="9"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorTitle="Phân loại không hợp lệ" error="Chọn 1 trong 5 phân loại có sẵn" sqref="D16:D39 C3:C39 D3:D7" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Phân loại không hợp lệ" error="Chọn 1 trong 5 phân loại có sẵn" sqref="D3:D8 C3:C16 C17:D33" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"An ninh mạng,Chuyển đổi số,Đổi mới sáng tạo,Nghiên cứu khoa học,Khác"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1448,6 +1731,17 @@
     <hyperlink ref="H3" r:id="rId1" xr:uid="{4828F916-DF36-6C4C-8558-FEA4D5FDB669}"/>
     <hyperlink ref="H4" r:id="rId2" xr:uid="{A7ECF054-C530-1845-B60B-097AE7F9D483}"/>
     <hyperlink ref="H5" r:id="rId3" xr:uid="{18E5B789-1E63-F642-9F4E-2D9E488140BD}"/>
+    <hyperlink ref="H16" r:id="rId4" xr:uid="{950D7AD0-3875-D742-BF32-206FFC45FC1E}"/>
+    <hyperlink ref="H12" r:id="rId5" xr:uid="{1D6236FD-EDE9-204D-B735-ED9C2100729A}"/>
+    <hyperlink ref="H10" r:id="rId6" xr:uid="{991E11A3-E531-3645-A17E-042F2D685967}"/>
+    <hyperlink ref="H9" r:id="rId7" xr:uid="{8C33CB3E-24FD-9743-B209-772ECD1B64B5}"/>
+    <hyperlink ref="H17" r:id="rId8" xr:uid="{166B5CE2-015D-884F-9BA0-97D88EEAFDFD}"/>
+    <hyperlink ref="H30" r:id="rId9" xr:uid="{1C8C8623-EE3F-B84D-A2C6-90F5890BC3E5}"/>
+    <hyperlink ref="H28" r:id="rId10" xr:uid="{C30DAB19-68BF-5140-AB20-7B55C7948F3A}"/>
+    <hyperlink ref="I8" r:id="rId11" xr:uid="{81789C96-391F-CB48-A5C8-52BFFE1FD79D}"/>
+    <hyperlink ref="H7" r:id="rId12" xr:uid="{6E63F5B3-8B2F-BA4E-A444-4E65AC4E78A0}"/>
+    <hyperlink ref="H18" r:id="rId13" xr:uid="{B596814D-D0DE-C041-9382-C89837C824BD}"/>
+    <hyperlink ref="H19" r:id="rId14" xr:uid="{99F4BCF6-49AF-4CA5-B401-56A9FF0365FC}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>